<commit_message>
Update: Remoção do arquivo de pré-processamento utilizando K-means
</commit_message>
<xml_diff>
--- a/docs/Especificações.xlsx
+++ b/docs/Especificações.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guilherme\Desktop\6º Semestre\TCC\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5D510D-112B-40CA-8879-08DF2CC553A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2CD059-5338-40C0-A5FF-08274CF2A2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{69908BCD-CF23-4C8B-B737-0A5881F10D2A}"/>
   </bookViews>
@@ -745,16 +745,16 @@
     <t>Tomato___Septoria_leaf_spot</t>
   </si>
   <si>
-    <t>Distribution of classes</t>
-  </si>
-  <si>
-    <t>Image quantity</t>
-  </si>
-  <si>
-    <t>Percentage</t>
-  </si>
-  <si>
     <t>Environment variables (PATH) added</t>
+  </si>
+  <si>
+    <t>Distribuição de classes</t>
+  </si>
+  <si>
+    <t>Qtd imagens</t>
+  </si>
+  <si>
+    <t>Percentual</t>
   </si>
 </sst>
 </file>
@@ -837,7 +837,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -847,6 +847,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1149,6 +1161,33 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1167,68 +1206,12 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1340,13 +1323,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1359,6 +1335,48 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -1375,12 +1393,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE62A65A-F5A0-433D-AD7F-01FC0E4909C9}" name="Tabela1" displayName="Tabela1" ref="B3:D14" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE62A65A-F5A0-433D-AD7F-01FC0E4909C9}" name="Tabela1" displayName="Tabela1" ref="B3:D14" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
   <autoFilter ref="B3:D14" xr:uid="{BE62A65A-F5A0-433D-AD7F-01FC0E4909C9}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{0577AAF6-2A51-4855-8024-F0F0B9CD76B0}" name="Distribution of classes" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{4B7B7387-D6FF-46CB-AC53-4BEA693BF93F}" name="Image quantity" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{532294A8-1A5C-4A77-B43A-3A814E3A58F6}" name="Percentage" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{0577AAF6-2A51-4855-8024-F0F0B9CD76B0}" name="Distribuição de classes" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{4B7B7387-D6FF-46CB-AC53-4BEA693BF93F}" name="Qtd imagens" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{532294A8-1A5C-4A77-B43A-3A814E3A58F6}" name="Percentual" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1713,10 +1731,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="C3" s="25"/>
+      <c r="C3" s="27"/>
     </row>
     <row r="4" spans="2:3" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="6" t="s">
@@ -1806,7 +1824,7 @@
     </row>
     <row r="22" spans="2:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="23" spans="2:2" s="18" customFormat="1" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1845,145 +1863,145 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="28" t="s">
-        <v>233</v>
-      </c>
-      <c r="C3" s="29" t="s">
+      <c r="B3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="C3" s="22" t="s">
         <v>235</v>
       </c>
+      <c r="D3" s="23" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="4" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="19" t="s">
         <v>222</v>
       </c>
       <c r="C4" s="17">
         <v>2127</v>
       </c>
-      <c r="D4" s="27">
-        <f>C4/$C$14</f>
+      <c r="D4" s="20">
+        <f t="shared" ref="D4:D13" si="0">C4/$C$14</f>
         <v>0.11712555066079296</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="19" t="s">
         <v>223</v>
       </c>
       <c r="C5" s="17">
         <v>1000</v>
       </c>
-      <c r="D5" s="27">
-        <f>C5/$C$14</f>
+      <c r="D5" s="20">
+        <f t="shared" si="0"/>
         <v>5.5066079295154183E-2</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="19" t="s">
         <v>224</v>
       </c>
       <c r="C6" s="17">
         <v>1909</v>
       </c>
-      <c r="D6" s="27">
-        <f>C6/$C$14</f>
+      <c r="D6" s="20">
+        <f t="shared" si="0"/>
         <v>0.10512114537444935</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="19" t="s">
         <v>225</v>
       </c>
       <c r="C7" s="17">
         <v>952</v>
       </c>
-      <c r="D7" s="27">
-        <f t="shared" ref="D7:D13" si="0">C7/$C$14</f>
+      <c r="D7" s="20">
+        <f t="shared" si="0"/>
         <v>5.2422907488986786E-2</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="19" t="s">
         <v>232</v>
       </c>
       <c r="C8" s="17">
         <v>1771</v>
       </c>
-      <c r="D8" s="27">
+      <c r="D8" s="20">
         <f t="shared" si="0"/>
         <v>9.7522026431718062E-2</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="19" t="s">
         <v>226</v>
       </c>
       <c r="C9" s="17">
         <v>1676</v>
       </c>
-      <c r="D9" s="27">
+      <c r="D9" s="20">
         <f t="shared" si="0"/>
         <v>9.2290748898678415E-2</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="19" t="s">
         <v>227</v>
       </c>
       <c r="C10" s="17">
         <v>1404</v>
       </c>
-      <c r="D10" s="27">
+      <c r="D10" s="20">
         <f t="shared" si="0"/>
         <v>7.7312775330396474E-2</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="19" t="s">
         <v>228</v>
       </c>
       <c r="C11" s="17">
         <v>5357</v>
       </c>
-      <c r="D11" s="27">
+      <c r="D11" s="20">
         <f t="shared" si="0"/>
         <v>0.29498898678414098</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="19" t="s">
         <v>229</v>
       </c>
       <c r="C12" s="17">
         <v>373</v>
       </c>
-      <c r="D12" s="27">
+      <c r="D12" s="20">
         <f t="shared" si="0"/>
         <v>2.053964757709251E-2</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="19" t="s">
         <v>230</v>
       </c>
       <c r="C13" s="17">
         <v>1591</v>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="20">
         <f t="shared" si="0"/>
         <v>8.7610132158590315E-2</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="24" t="s">
         <v>231</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="25">
         <f>SUM(C4:C13)</f>
         <v>18160</v>
       </c>
-      <c r="D14" s="33">
+      <c r="D14" s="26">
         <f>SUM(D4:D13)</f>
         <v>1</v>
       </c>
@@ -2011,27 +2029,27 @@
     </row>
     <row r="3" spans="3:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="21"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="30"/>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="3:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C5" s="22"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="24"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="33"/>
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="3:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>